<commit_message>
QC-centred PCA (compounds without imputed values), 11-oxoetiocholanolone glucuronide annotation (no double counting with THE glucuronide), imputed values as open symbols, axis wording; run_all keeps results/blank_check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/publication_v4/figures_tables/Tables_main.xlsx
+++ b/publication_v4/figures_tables/Tables_main.xlsx
@@ -767,7 +767,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C19H28O3 oxo-androstane (putatively 11-oxoetiocholanolone)</t>
+          <t>11-Oxoetiocholanolone glucuronide (putative)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>C19H28O3 steroid isomers (e.g., 11-oxoetiocholanolone, 11-oxoandrosterone, 7β-hydroxy-DHEA) not resolved</t>
+          <t>11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -1213,7 +1213,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Isomers: C19H28O3 oxo-androstane (putatively 11-oxoetiocholanolone): C19H28O3 steroid isomers (e.g., 11-oxoetiocholanolone, 11-oxoandrosterone, 7β-hydroxy-DHEA) not resolved; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Dodecanoylcarnitine: branched-chain C12 acylcarnitine isomers not excluded; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Valyl-Leucine: Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
+          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Dodecanoylcarnitine: branched-chain C12 acylcarnitine isomers not excluded; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Valyl-Leucine: Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Table 2: library match of the aglycone ion for the steroid glucuronides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/publication_v4/figures_tables/Tables_main.xlsx
+++ b/publication_v4/figures_tables/Tables_main.xlsx
@@ -772,7 +772,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5.beta.-Androstan-3.alpha.-ol-11,17-dione</t>
+          <t>5.beta.-Androstan-3.alpha.-ol-11,17-dione (11-oxoetiocholanolone; MS/MS of the aglycone ion)</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -835,7 +835,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NCGC00380230-01_C26H40O9_2,4a,6-Trihydroxy-8-isopropyl-1,1-dimethyl-2,3,4,4a,5,10,11,11a-octahydro-1H-dibenzo[a,d][7]annulen-7-yl beta-D-glucopyranoside</t>
+          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -961,7 +961,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
         </is>
       </c>
       <c r="D5" t="n">

</xml_diff>

<commit_message>
Compound representative = curated intact-molecule ion when present (11-oxoetiocholanolone glucuronide now on m/z 498.2697); imputation sensitivity analysis (Table S7); confirmation of the 10.76-min tetrahydrocortisone glucuronide isomer; texts updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/publication_v4/figures_tables/Tables_main.xlsx
+++ b/publication_v4/figures_tables/Tables_main.xlsx
@@ -776,17 +776,17 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>287.2007</v>
+        <v>498.2697</v>
       </c>
       <c r="E2" t="n">
-        <v>11.06</v>
+        <v>11.05</v>
       </c>
       <c r="F2" t="n">
         <v>3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -798,15 +798,15 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1.25</v>
+        <v>1.49</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>6.3e-03</t>
+          <t>5.6e-03</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ages/sex updated for controls 20, 62, 94; full recalculation (222 findings, 20 BC-control and 11 PC-control pairs; Table 2 now 6 compounds), submission text updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/publication_v4/figures_tables/Tables_main.xlsx
+++ b/publication_v4/figures_tables/Tables_main.xlsx
@@ -460,21 +460,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>18/25 (2)</t>
+          <t>19/26 (0)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>53.3 ± 13.9</t>
+          <t>53.0 ± 14.9</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>58 (25–72)</t>
+          <t>58 (18–72)</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -544,7 +544,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Age was not available for 4 participants (4 Control) and sex for 2 (2 Control); 0 lacked both. These participants were retained in the unadjusted analyses (Mann–Whitney U tests, exogenous-signal index, cross-validated models on all samples) and excluded from the adjusted linear model (complete-case analysis, n = 88 of 94) and from age- and index-matched pairs; missing values were not imputed.</t>
+          <t>Age was not available for 3 participants (3 Control) and sex for 0 (); 0 lacked both. These participants were retained in the unadjusted analyses (Mann–Whitney U tests, exogenous-signal index, cross-validated models on all samples) and excluded from the adjusted linear model (complete-case analysis, n = 91 of 94) and from age- and index-matched pairs; missing values were not imputed.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2.3e-06</t>
+          <t>3.1e-06</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.0057</t>
+          <t>0.0067</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.00064</t>
+          <t>0.00068</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.2e-06</t>
+          <t>1.7e-06</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.2e-06</t>
+          <t>3.5e-06</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8.2e-05</t>
+          <t>7.7e-05</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -798,11 +798,11 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1.49</v>
+        <v>1.42</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.6e-03</t>
+          <t>5.9e-03</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -810,7 +810,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1.14</v>
+        <v>1.06</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.9e-02</t>
+          <t>2.3e-02</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -873,7 +873,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0.011</t>
+          <t>0.026</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -893,19 +893,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dodecanoylcarnitine</t>
+          <t>LysoPC(16:0)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LAUROYLCARNITINE</t>
+          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>344.2797</v>
+        <v>496.3397</v>
       </c>
       <c r="E4" t="n">
-        <v>14.37</v>
+        <v>16.71</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -920,33 +920,33 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>branched-chain C12 acylcarnitine isomers not excluded</t>
+          <t>sn-1/sn-2 regioisomers not resolved</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.93</v>
+        <v>1.33</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.0e-02</t>
+          <t>3.0e-02</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.73</v>
+        <v>0.79</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.045</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>100/97/100</t>
+          <t>100/100/100</t>
         </is>
       </c>
     </row>
@@ -956,60 +956,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tetrahydrocortisone glucuronide (putative)</t>
+          <t>Biliverdin</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
+          <t>BILIVERDIN</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>558.2914</v>
+        <v>583.2553</v>
       </c>
       <c r="E5" t="n">
-        <v>10.76</v>
+        <v>13.48</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
+          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.87</v>
+        <v>2.2</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.9e-02</t>
+          <t>3.1e-02</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.77</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.045</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.019</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>100/100/100</t>
+          <t>89/97/75</t>
         </is>
       </c>
     </row>
@@ -1019,60 +1019,60 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Biliverdin</t>
+          <t>Tetrahydrocortisone glucuronide (putative)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BILIVERDIN</t>
+          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>583.2553</v>
+        <v>558.2914</v>
       </c>
       <c r="E6" t="n">
-        <v>13.48</v>
+        <v>10.76</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
+          <t>tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2.18</v>
+        <v>0.8</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.3e-02</t>
+          <t>3.7e-02</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.77</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0.046</t>
+          <t>0.021</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.019</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>89/97/75</t>
+          <t>100/100/100</t>
         </is>
       </c>
     </row>
@@ -1082,19 +1082,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LysoPC(16:0)</t>
+          <t>Valyl-Leucine</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
+          <t>Val-Leu</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>496.3397</v>
+        <v>231.1704</v>
       </c>
       <c r="E7" t="n">
-        <v>16.71</v>
+        <v>3.72</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -1109,111 +1109,48 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>sn-1/sn-2 regioisomers not resolved</t>
+          <t>Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1.3</v>
+        <v>1.68</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.4e-02</t>
+          <t>3.9e-02</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.79</v>
+        <v>0.76</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0.005</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>100/100/100</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Valyl-Leucine</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Val-Leu</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>231.1704</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>4.8e-02</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>0.004</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0.001</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
           <t>98/100/100</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Dodecanoylcarnitine: branched-chain C12 acylcarnitine isomers not excluded; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Valyl-Leucine: Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
+          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Valyl-Leucine: Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ages for controls 15, 25, 72 added (no missing age/sex); full recalculation: 210 findings, Table 2 with 5 compounds; submission text updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/publication_v4/figures_tables/Tables_main.xlsx
+++ b/publication_v4/figures_tables/Tables_main.xlsx
@@ -465,16 +465,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>53.0 ± 14.9</t>
+          <t>53.3 ± 14.6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>58 (18–72)</t>
+          <t>59 (18–72)</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -544,7 +544,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Age was not available for 3 participants (3 Control). These participants were retained in the unadjusted analyses (Mann–Whitney U tests, exogenous-signal index, cross-validated models on all samples) and excluded from the adjusted linear model (complete-case analysis, n = 91 of 94) and from age-matched pairs; missing values were not imputed.</t>
+          <t>Age and sex were available for all participants.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3.1e-06</t>
+          <t>2e-06</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.0067</t>
+          <t>0.0072</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.7e-06</t>
+          <t>9.2e-07</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -798,11 +798,11 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.9e-03</t>
+          <t>4.7e-03</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.3e-02</t>
+          <t>1.8e-02</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -893,19 +893,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LysoPC(16:0)</t>
+          <t>Biliverdin</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
+          <t>BILIVERDIN</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>496.3397</v>
+        <v>583.2553</v>
       </c>
       <c r="E4" t="n">
-        <v>16.71</v>
+        <v>13.48</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -920,33 +920,33 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>sn-1/sn-2 regioisomers not resolved</t>
+          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1.33</v>
+        <v>2.23</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>3.0e-02</t>
+          <t>2.4e-02</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.003</t>
+          <t>0.042</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>100/100/100</t>
+          <t>89/97/75</t>
         </is>
       </c>
     </row>
@@ -956,19 +956,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Biliverdin</t>
+          <t>LysoPC(16:0)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BILIVERDIN</t>
+          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>583.2553</v>
+        <v>496.3397</v>
       </c>
       <c r="E5" t="n">
-        <v>13.48</v>
+        <v>16.71</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -983,33 +983,33 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
+          <t>sn-1/sn-2 regioisomers not resolved</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2.2</v>
+        <v>1.33</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.1e-02</t>
+          <t>2.5e-02</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.045</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>89/97/75</t>
+          <t>100/100/100</t>
         </is>
       </c>
     </row>
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>3.7e-02</t>
+          <t>3.0e-02</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0.021</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1076,81 +1076,18 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Valyl-Leucine</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Val-Leu</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>231.1704</v>
-      </c>
-      <c r="E7" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>3.9e-02</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>0.008</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0.001</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>98/100/100</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Valyl-Leucine: Leu-Val, Val-Ile and Ile-Val not excluded by MS/MS; in this dataset MS-DIAL also matched Leu-Val (2.68 min) and Val-Leu (3.93 min) at the same m/z</t>
+          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
         </is>
       </c>
     </row>

</xml_diff>